<commit_message>
Harden commands and model loading
Tightens several viewer and MCP behaviors: metadata filters now support negative numeric ranges, `color` rejects invalid scales, `label` parses `%` thresholds correctly, `select save` is restricted to the leading form, `spectrum` treats infinities as invalid, and command-catalog help extraction now preserves full f-strings and alternate usage lines.

It also improves runtime/config handling by surfacing unavailable saved embedding models in the Tools UI, rejecting 3D caches in the desktop viewer with a clearer error, validating `start_layout_job` parameter keys, narrowing ESMFold local data-root overrides to ESM3, and removing the unused ESM-2 pooler while only hiding non-actionable Transformers load reports. Related docs and tests were updated to match.
</commit_message>
<xml_diff>
--- a/docs/metadata_template.xlsx
+++ b/docs/metadata_template.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/xuebin_feng_mail_utoronto_ca/Documents/Research Records/Computational Methods/Sequence_Similarity_Network_Viewer/docs/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="11" documentId="11_3C77112C777A147E4738FC623260F5DBC8C596C2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68BE3A06-B4D5-405B-83C9-B831A575254A}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>

<commit_message>
Reserve only canonical subcluster labels
Generated subcluster labels are now limited to canonical names with positive integer IDs and no leading zeros. `subcluster clear` removes only those generated labels while preserving custom lookalikes such as `subcluster_0_2` and `subcluster_001_2`, and re-running `subcluster cluster_N` replaces only the generated labels for that cluster. Documentation and tests were updated to reflect the new reserved-name behavior.
</commit_message>
<xml_diff>
--- a/docs/metadata_template.xlsx
+++ b/docs/metadata_template.xlsx
@@ -746,10 +746,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{78aac226-2f03-4b4d-9037-b46d56c55210}" enabled="0" method="" siteId="{78aac226-2f03-4b4d-9037-b46d56c55210}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>